<commit_message>
Added file download utlity
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
@@ -519,7 +519,7 @@
         <v>95.221075283944316</v>
       </c>
       <c r="E2" s="2">
-        <v>129.84966844900714</v>
+        <v>129.84966844900711</v>
       </c>
     </row>
     <row r="3">
@@ -533,10 +533,10 @@
         <v>2011</v>
       </c>
       <c r="D3" s="2">
-        <v>86.955464237230856</v>
+        <v>86.955464237230871</v>
       </c>
       <c r="E3" s="2">
-        <v>123.95548470731528</v>
+        <v>123.95548470731531</v>
       </c>
     </row>
     <row r="4">
@@ -550,10 +550,10 @@
         <v>2012</v>
       </c>
       <c r="D4" s="2">
-        <v>83.958370647084877</v>
+        <v>83.958370647084891</v>
       </c>
       <c r="E4" s="2">
-        <v>125.98492039902339</v>
+        <v>125.98492039902337</v>
       </c>
     </row>
     <row r="5">
@@ -604,7 +604,7 @@
         <v>102.44156425394573</v>
       </c>
       <c r="E7" s="2">
-        <v>123.99215185512162</v>
+        <v>123.99215185512165</v>
       </c>
     </row>
     <row r="8">
@@ -652,10 +652,10 @@
         <v>2018</v>
       </c>
       <c r="D10" s="2">
-        <v>107.65095729890695</v>
+        <v>107.65095729890692</v>
       </c>
       <c r="E10" s="2">
-        <v>134.91772827836096</v>
+        <v>134.91772827836098</v>
       </c>
     </row>
     <row r="11">
@@ -672,7 +672,7 @@
         <v>119.09170030342355</v>
       </c>
       <c r="E11" s="2">
-        <v>144.1067785803204</v>
+        <v>144.10677858032042</v>
       </c>
     </row>
     <row r="12">
@@ -706,7 +706,7 @@
         <v>98.03239321958435</v>
       </c>
       <c r="E13" s="2">
-        <v>126.94754679620044</v>
+        <v>126.94754679620046</v>
       </c>
     </row>
     <row r="14">
@@ -720,7 +720,7 @@
         <v>2022</v>
       </c>
       <c r="D14" s="2">
-        <v>106.17568685241636</v>
+        <v>106.17568685241639</v>
       </c>
       <c r="E14" s="2">
         <v>136.01723072341716</v>
@@ -771,7 +771,7 @@
         <v>2011</v>
       </c>
       <c r="D17" s="2">
-        <v>109.30850739434268</v>
+        <v>109.30850739434271</v>
       </c>
       <c r="E17" s="2">
         <v>155.36787412863711</v>
@@ -805,7 +805,7 @@
         <v>2013</v>
       </c>
       <c r="D19" s="2">
-        <v>153.29967899492223</v>
+        <v>153.29967899492226</v>
       </c>
       <c r="E19" s="2">
         <v>188.36042775237485</v>
@@ -825,7 +825,7 @@
         <v>125.33096468512295</v>
       </c>
       <c r="E20" s="2">
-        <v>151.69288037849711</v>
+        <v>151.69288037849714</v>
       </c>
     </row>
     <row r="21">
@@ -842,7 +842,7 @@
         <v>126.40360469611636</v>
       </c>
       <c r="E21" s="2">
-        <v>147.36292080522935</v>
+        <v>147.36292080522929</v>
       </c>
     </row>
     <row r="22">
@@ -856,7 +856,7 @@
         <v>2016</v>
       </c>
       <c r="D22" s="2">
-        <v>141.21050447640189</v>
+        <v>141.21050447640192</v>
       </c>
       <c r="E22" s="2">
         <v>178.69433588102015</v>
@@ -893,7 +893,7 @@
         <v>143.09130434286234</v>
       </c>
       <c r="E24" s="2">
-        <v>171.99142090267486</v>
+        <v>171.99142090267489</v>
       </c>
     </row>
     <row r="25">
@@ -924,7 +924,7 @@
         <v>2020</v>
       </c>
       <c r="D26" s="2">
-        <v>139.3940110249097</v>
+        <v>139.39401102490973</v>
       </c>
       <c r="E26" s="2">
         <v>169.28851560092858</v>
@@ -941,7 +941,7 @@
         <v>2021</v>
       </c>
       <c r="D27" s="2">
-        <v>133.04510412862652</v>
+        <v>133.04510412862646</v>
       </c>
       <c r="E27" s="2">
         <v>166.87172048037422</v>
@@ -958,7 +958,7 @@
         <v>2022</v>
       </c>
       <c r="D28" s="2">
-        <v>135.55051913987518</v>
+        <v>135.55051913987521</v>
       </c>
       <c r="E28" s="2">
         <v>187.12143427741452</v>
@@ -975,7 +975,7 @@
         <v>2023</v>
       </c>
       <c r="D29" s="2">
-        <v>153.96482802987171</v>
+        <v>153.96482802987174</v>
       </c>
       <c r="E29" s="2">
         <v>197.85764950643474</v>
@@ -1012,7 +1012,7 @@
         <v>97.059790074554726</v>
       </c>
       <c r="E31" s="2">
-        <v>138.75412658257852</v>
+        <v>138.75412658257849</v>
       </c>
     </row>
     <row r="32">
@@ -1026,7 +1026,7 @@
         <v>2012</v>
       </c>
       <c r="D32" s="2">
-        <v>97.496314274191278</v>
+        <v>97.496314274191263</v>
       </c>
       <c r="E32" s="2">
         <v>137.91417726388366</v>
@@ -1063,7 +1063,7 @@
         <v>115.29448083495107</v>
       </c>
       <c r="E34" s="2">
-        <v>137.41944314066933</v>
+        <v>137.41944314066939</v>
       </c>
     </row>
     <row r="35">
@@ -1097,7 +1097,7 @@
         <v>131.85208906168819</v>
       </c>
       <c r="E36" s="2">
-        <v>166.16480818173736</v>
+        <v>166.16480818173733</v>
       </c>
     </row>
     <row r="37">
@@ -1111,10 +1111,10 @@
         <v>2017</v>
       </c>
       <c r="D37" s="2">
-        <v>124.35262647776938</v>
+        <v>124.35262647776935</v>
       </c>
       <c r="E37" s="2">
-        <v>146.69798774634043</v>
+        <v>146.69798774634046</v>
       </c>
     </row>
     <row r="38">
@@ -1128,10 +1128,10 @@
         <v>2018</v>
       </c>
       <c r="D38" s="2">
-        <v>124.24670561488776</v>
+        <v>124.24670561488777</v>
       </c>
       <c r="E38" s="2">
-        <v>152.43280946429914</v>
+        <v>152.43280946429917</v>
       </c>
     </row>
     <row r="39">
@@ -1162,7 +1162,7 @@
         <v>2020</v>
       </c>
       <c r="D40" s="2">
-        <v>124.30445543196633</v>
+        <v>124.30445543196635</v>
       </c>
       <c r="E40" s="2">
         <v>152.29672324055017</v>
@@ -1179,7 +1179,7 @@
         <v>2021</v>
       </c>
       <c r="D41" s="2">
-        <v>113.58524224366188</v>
+        <v>113.5852422436619</v>
       </c>
       <c r="E41" s="2">
         <v>144.70940452701333</v>
@@ -1199,7 +1199,7 @@
         <v>119.57775610158743</v>
       </c>
       <c r="E42" s="2">
-        <v>158.71716158231379</v>
+        <v>158.71716158231376</v>
       </c>
     </row>
     <row r="43">
@@ -1213,7 +1213,7 @@
         <v>2023</v>
       </c>
       <c r="D43" s="2">
-        <v>130.35018720620911</v>
+        <v>130.35018720620914</v>
       </c>
       <c r="E43" s="2">
         <v>166.47644866986056</v>
@@ -1250,7 +1250,7 @@
         <v>20.736462077997842</v>
       </c>
       <c r="E45" s="2">
-        <v>50.7496704331015</v>
+        <v>50.749670433101471</v>
       </c>
     </row>
     <row r="46">
@@ -1264,10 +1264,10 @@
         <v>2012</v>
       </c>
       <c r="D46" s="2">
-        <v>40.861820365951232</v>
+        <v>40.861820365951246</v>
       </c>
       <c r="E46" s="2">
-        <v>80.862069789296086</v>
+        <v>80.862069789296101</v>
       </c>
     </row>
     <row r="47">
@@ -1298,10 +1298,10 @@
         <v>2014</v>
       </c>
       <c r="D48" s="2">
-        <v>44.404040284993002</v>
+        <v>44.404040284992988</v>
       </c>
       <c r="E48" s="2">
-        <v>72.287202202189931</v>
+        <v>72.287202202189945</v>
       </c>
     </row>
     <row r="49">
@@ -1437,7 +1437,7 @@
         <v>38.830144120011511</v>
       </c>
       <c r="E56" s="2">
-        <v>87.948672510579129</v>
+        <v>87.948672510579144</v>
       </c>
     </row>
     <row r="57">
@@ -1454,7 +1454,7 @@
         <v>38.436967798230711</v>
       </c>
       <c r="E57" s="2">
-        <v>89.923140516683503</v>
+        <v>89.923140516683517</v>
       </c>
     </row>
     <row r="58">
@@ -1502,10 +1502,10 @@
         <v>2012</v>
       </c>
       <c r="D60" s="2">
-        <v>53.267849983925771</v>
+        <v>53.267849983925743</v>
       </c>
       <c r="E60" s="2">
-        <v>119.72367489464595</v>
+        <v>119.72367489464597</v>
       </c>
     </row>
     <row r="61">
@@ -1539,7 +1539,7 @@
         <v>70.396366189709895</v>
       </c>
       <c r="E62" s="2">
-        <v>124.02873729314173</v>
+        <v>124.02873729314176</v>
       </c>
     </row>
     <row r="63">
@@ -1553,10 +1553,10 @@
         <v>2015</v>
       </c>
       <c r="D63" s="2">
-        <v>63.096850001600338</v>
+        <v>63.096850001600352</v>
       </c>
       <c r="E63" s="2">
-        <v>95.253253760130406</v>
+        <v>95.253253760130392</v>
       </c>
     </row>
     <row r="64">
@@ -1573,7 +1573,7 @@
         <v>67.298402962039859</v>
       </c>
       <c r="E64" s="2">
-        <v>136.09138427814995</v>
+        <v>136.09138427814997</v>
       </c>
     </row>
     <row r="65">
@@ -1590,7 +1590,7 @@
         <v>77.910922958684793</v>
       </c>
       <c r="E65" s="2">
-        <v>134.62413985681277</v>
+        <v>134.6241398568128</v>
       </c>
     </row>
     <row r="66">
@@ -1607,7 +1607,7 @@
         <v>79.962100676298675</v>
       </c>
       <c r="E66" s="2">
-        <v>142.28837093119802</v>
+        <v>142.28837093119805</v>
       </c>
     </row>
     <row r="67">
@@ -1621,10 +1621,10 @@
         <v>2019</v>
       </c>
       <c r="D67" s="2">
-        <v>82.511839058747782</v>
+        <v>82.511839058747768</v>
       </c>
       <c r="E67" s="2">
-        <v>140.53768006006936</v>
+        <v>140.53768006006933</v>
       </c>
     </row>
     <row r="68">
@@ -1638,7 +1638,7 @@
         <v>2020</v>
       </c>
       <c r="D68" s="2">
-        <v>84.746575532747755</v>
+        <v>84.746575532747769</v>
       </c>
       <c r="E68" s="2">
         <v>146.62608239079285</v>
@@ -1672,10 +1672,10 @@
         <v>2022</v>
       </c>
       <c r="D70" s="2">
-        <v>65.485466952983003</v>
+        <v>65.485466952982989</v>
       </c>
       <c r="E70" s="2">
-        <v>153.94379226746622</v>
+        <v>153.94379226746625</v>
       </c>
     </row>
     <row r="71">
@@ -1689,10 +1689,10 @@
         <v>2023</v>
       </c>
       <c r="D71" s="2">
-        <v>67.995052411881915</v>
+        <v>67.995052411881929</v>
       </c>
       <c r="E71" s="2">
-        <v>144.77017142602571</v>
+        <v>144.77017142602574</v>
       </c>
     </row>
     <row r="72">
@@ -1709,7 +1709,7 @@
         <v>32.859156905523491</v>
       </c>
       <c r="E72" s="2">
-        <v>85.93946563238552</v>
+        <v>85.939465632385506</v>
       </c>
     </row>
     <row r="73">
@@ -1743,7 +1743,7 @@
         <v>46.493243333067454</v>
       </c>
       <c r="E74" s="2">
-        <v>98.372077995995952</v>
+        <v>98.372077995995923</v>
       </c>
     </row>
     <row r="75">
@@ -1777,7 +1777,7 @@
         <v>56.098523893632731</v>
       </c>
       <c r="E76" s="2">
-        <v>95.203378791033103</v>
+        <v>95.203378791033131</v>
       </c>
     </row>
     <row r="77">
@@ -1791,7 +1791,7 @@
         <v>2015</v>
       </c>
       <c r="D77" s="2">
-        <v>51.214620843783862</v>
+        <v>51.214620843783848</v>
       </c>
       <c r="E77" s="2">
         <v>76.650630627800695</v>
@@ -1845,7 +1845,7 @@
         <v>58.275368982340389</v>
       </c>
       <c r="E80" s="2">
-        <v>106.8477281211683</v>
+        <v>106.84772812116829</v>
       </c>
     </row>
     <row r="81">
@@ -1879,7 +1879,7 @@
         <v>62.987702944194631</v>
       </c>
       <c r="E82" s="2">
-        <v>116.7731476771192</v>
+        <v>116.77314767711917</v>
       </c>
     </row>
     <row r="83">

</xml_diff>

<commit_message>
Formatted latest tabulations page (tables 1-7)
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="396" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="396" uniqueCount="115">
   <si>
     <t>field</t>
   </si>
@@ -282,25 +282,40 @@
     <t>CVD in Men (vs. Women)</t>
   </si>
   <si>
-    <t>2012-2013 (vs. 2010-11)</t>
-  </si>
-  <si>
-    <t>2014-2015</t>
-  </si>
-  <si>
-    <t>2016-2017</t>
-  </si>
-  <si>
-    <t>2018-2019</t>
-  </si>
-  <si>
-    <t>2020-2021</t>
-  </si>
-  <si>
-    <t>2022-2023</t>
-  </si>
-  <si>
-    <t>2012-2013</t>
+    <t>Stroke&lt;br&gt;2012-2013 (vs. 2010-11)</t>
+  </si>
+  <si>
+    <t>Stroke&lt;br&gt;2014-2015</t>
+  </si>
+  <si>
+    <t>Stroke&lt;br&gt;2016-2017</t>
+  </si>
+  <si>
+    <t>Stroke&lt;br&gt;2018-2019</t>
+  </si>
+  <si>
+    <t>Stroke&lt;br&gt;2020-2021</t>
+  </si>
+  <si>
+    <t>Stroke&lt;br&gt;2022-2023</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2012-2013</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2014-2015</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2016-2017</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2018-2019</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2020-2021</t>
+  </si>
+  <si>
+    <t>AMI&lt;br&gt;2022-2023</t>
   </si>
   <si>
     <t>srr</t>
@@ -327,7 +342,7 @@
     <t>Based on hospital CVD event only</t>
   </si>
   <si>
-    <t>%23.0g</t>
+    <t>%33.0g</t>
   </si>
   <si>
     <t>%5.3f</t>
@@ -348,7 +363,7 @@
     <t>Upper bound of SRR</t>
   </si>
   <si>
-    <t xml:space="preserve">1=Stroke (vs. AMI); 2=CVD in Men (vs. Women); 4=2012-2013 (vs. 2010-11); 5=2014-2015; 6=2016-2017; 7=2018-2019; 8=2020-2021; 9=2022-2023; 11=2012-2013; 12=2014-2015; 13=2016-2017; 14=2018-2019; 15=2020-2021; 16=2022-2023; </t>
+    <t xml:space="preserve">1=Stroke (vs. AMI); 2=CVD in Men (vs. Women); 4=Stroke&lt;br&gt;2012-2013 (vs. 2010-11); 5=Stroke&lt;br&gt;2014-2015; 6=Stroke&lt;br&gt;2016-2017; 7=Stroke&lt;br&gt;2018-2019; 8=Stroke&lt;br&gt;2020-2021; 9=Stroke&lt;br&gt;2022-2023; 11=AMI&lt;br&gt;2012-2013; 12=AMI&lt;br&gt;2014-2015; 13=AMI&lt;br&gt;2016-2017; 14=AMI&lt;br&gt;2018-2019; 15=AMI&lt;br&gt;2020-2021; 16=AMI&lt;br&gt;2022-2023; </t>
   </si>
 </sst>
 </file>
@@ -536,7 +551,7 @@
         <v>86.955464237230871</v>
       </c>
       <c r="E3" s="2">
-        <v>123.95548470731531</v>
+        <v>123.95548470731534</v>
       </c>
     </row>
     <row r="4">
@@ -550,7 +565,7 @@
         <v>2012</v>
       </c>
       <c r="D4" s="2">
-        <v>83.958370647084891</v>
+        <v>83.958370647084877</v>
       </c>
       <c r="E4" s="2">
         <v>125.98492039902337</v>
@@ -587,7 +602,7 @@
         <v>106.6020394396615</v>
       </c>
       <c r="E6" s="2">
-        <v>126.50748443185483</v>
+        <v>126.50748443185482</v>
       </c>
     </row>
     <row r="7">
@@ -601,7 +616,7 @@
         <v>2015</v>
       </c>
       <c r="D7" s="2">
-        <v>102.44156425394573</v>
+        <v>102.44156425394576</v>
       </c>
       <c r="E7" s="2">
         <v>123.99215185512165</v>
@@ -638,7 +653,7 @@
         <v>113.46297582983944</v>
       </c>
       <c r="E9" s="2">
-        <v>134.09629973602566</v>
+        <v>134.09629973602568</v>
       </c>
     </row>
     <row r="10">
@@ -655,7 +670,7 @@
         <v>107.65095729890692</v>
       </c>
       <c r="E10" s="2">
-        <v>134.91772827836098</v>
+        <v>134.91772827836096</v>
       </c>
     </row>
     <row r="11">
@@ -771,10 +786,10 @@
         <v>2011</v>
       </c>
       <c r="D17" s="2">
-        <v>109.30850739434271</v>
+        <v>109.30850739434268</v>
       </c>
       <c r="E17" s="2">
-        <v>155.36787412863711</v>
+        <v>155.36787412863708</v>
       </c>
     </row>
     <row r="18">
@@ -788,7 +803,7 @@
         <v>2012</v>
       </c>
       <c r="D18" s="2">
-        <v>114.55911018767614</v>
+        <v>114.55911018767617</v>
       </c>
       <c r="E18" s="2">
         <v>150.37591834701553</v>
@@ -805,7 +820,7 @@
         <v>2013</v>
       </c>
       <c r="D19" s="2">
-        <v>153.29967899492226</v>
+        <v>153.29967899492223</v>
       </c>
       <c r="E19" s="2">
         <v>188.36042775237485</v>
@@ -822,7 +837,7 @@
         <v>2014</v>
       </c>
       <c r="D20" s="2">
-        <v>125.33096468512295</v>
+        <v>125.33096468512296</v>
       </c>
       <c r="E20" s="2">
         <v>151.69288037849714</v>
@@ -842,7 +857,7 @@
         <v>126.40360469611636</v>
       </c>
       <c r="E21" s="2">
-        <v>147.36292080522929</v>
+        <v>147.36292080522932</v>
       </c>
     </row>
     <row r="22">
@@ -893,7 +908,7 @@
         <v>143.09130434286234</v>
       </c>
       <c r="E24" s="2">
-        <v>171.99142090267489</v>
+        <v>171.99142090267486</v>
       </c>
     </row>
     <row r="25">
@@ -924,7 +939,7 @@
         <v>2020</v>
       </c>
       <c r="D26" s="2">
-        <v>139.39401102490973</v>
+        <v>139.3940110249097</v>
       </c>
       <c r="E26" s="2">
         <v>169.28851560092858</v>
@@ -941,7 +956,7 @@
         <v>2021</v>
       </c>
       <c r="D27" s="2">
-        <v>133.04510412862646</v>
+        <v>133.04510412862652</v>
       </c>
       <c r="E27" s="2">
         <v>166.87172048037422</v>
@@ -961,7 +976,7 @@
         <v>135.55051913987521</v>
       </c>
       <c r="E28" s="2">
-        <v>187.12143427741452</v>
+        <v>187.12143427741455</v>
       </c>
     </row>
     <row r="29">
@@ -975,7 +990,7 @@
         <v>2023</v>
       </c>
       <c r="D29" s="2">
-        <v>153.96482802987174</v>
+        <v>153.96482802987171</v>
       </c>
       <c r="E29" s="2">
         <v>197.85764950643474</v>
@@ -992,7 +1007,7 @@
         <v>2010</v>
       </c>
       <c r="D30" s="2">
-        <v>108.19131887864872</v>
+        <v>108.1913188786487</v>
       </c>
       <c r="E30" s="2">
         <v>143.76442335625933</v>
@@ -1029,7 +1044,7 @@
         <v>97.496314274191263</v>
       </c>
       <c r="E32" s="2">
-        <v>137.91417726388366</v>
+        <v>137.91417726388363</v>
       </c>
     </row>
     <row r="33">
@@ -1043,7 +1058,7 @@
         <v>2013</v>
       </c>
       <c r="D33" s="2">
-        <v>132.43103487164558</v>
+        <v>132.43103487164561</v>
       </c>
       <c r="E33" s="2">
         <v>165.76438905854454</v>
@@ -1063,7 +1078,7 @@
         <v>115.29448083495107</v>
       </c>
       <c r="E34" s="2">
-        <v>137.41944314066939</v>
+        <v>137.41944314066936</v>
       </c>
     </row>
     <row r="35">
@@ -1077,10 +1092,10 @@
         <v>2015</v>
       </c>
       <c r="D35" s="2">
-        <v>113.84661645574478</v>
+        <v>113.84661645574481</v>
       </c>
       <c r="E35" s="2">
-        <v>135.50382164638725</v>
+        <v>135.50382164638728</v>
       </c>
     </row>
     <row r="36">
@@ -1097,7 +1112,7 @@
         <v>131.85208906168819</v>
       </c>
       <c r="E36" s="2">
-        <v>166.16480818173733</v>
+        <v>166.1648081817373</v>
       </c>
     </row>
     <row r="37">
@@ -1111,10 +1126,10 @@
         <v>2017</v>
       </c>
       <c r="D37" s="2">
-        <v>124.35262647776935</v>
+        <v>124.35262647776932</v>
       </c>
       <c r="E37" s="2">
-        <v>146.69798774634046</v>
+        <v>146.69798774634043</v>
       </c>
     </row>
     <row r="38">
@@ -1165,7 +1180,7 @@
         <v>124.30445543196635</v>
       </c>
       <c r="E40" s="2">
-        <v>152.29672324055017</v>
+        <v>152.29672324055014</v>
       </c>
     </row>
     <row r="41">
@@ -1196,7 +1211,7 @@
         <v>2022</v>
       </c>
       <c r="D42" s="2">
-        <v>119.57775610158743</v>
+        <v>119.5777561015874</v>
       </c>
       <c r="E42" s="2">
         <v>158.71716158231376</v>
@@ -1233,7 +1248,7 @@
         <v>26.751842023372774</v>
       </c>
       <c r="E44" s="2">
-        <v>73.478827397940265</v>
+        <v>73.478827397940279</v>
       </c>
     </row>
     <row r="45">
@@ -1264,10 +1279,10 @@
         <v>2012</v>
       </c>
       <c r="D46" s="2">
-        <v>40.861820365951246</v>
+        <v>40.861820365951232</v>
       </c>
       <c r="E46" s="2">
-        <v>80.862069789296101</v>
+        <v>80.862069789296086</v>
       </c>
     </row>
     <row r="47">
@@ -1301,7 +1316,7 @@
         <v>44.404040284992988</v>
       </c>
       <c r="E48" s="2">
-        <v>72.287202202189945</v>
+        <v>72.28720220218996</v>
       </c>
     </row>
     <row r="49">
@@ -1369,7 +1384,7 @@
         <v>40.85685773962669</v>
       </c>
       <c r="E52" s="2">
-        <v>77.837349073280748</v>
+        <v>77.837349073280763</v>
       </c>
     </row>
     <row r="53">
@@ -1420,7 +1435,7 @@
         <v>34.016850240943995</v>
       </c>
       <c r="E55" s="2">
-        <v>76.494922085252966</v>
+        <v>76.494922085252981</v>
       </c>
     </row>
     <row r="56">
@@ -1437,7 +1452,7 @@
         <v>38.830144120011511</v>
       </c>
       <c r="E56" s="2">
-        <v>87.948672510579144</v>
+        <v>87.948672510579129</v>
       </c>
     </row>
     <row r="57">
@@ -1454,7 +1469,7 @@
         <v>38.436967798230711</v>
       </c>
       <c r="E57" s="2">
-        <v>89.923140516683517</v>
+        <v>89.923140516683503</v>
       </c>
     </row>
     <row r="58">
@@ -1536,10 +1551,10 @@
         <v>2014</v>
       </c>
       <c r="D62" s="2">
-        <v>70.396366189709895</v>
+        <v>70.39636618970988</v>
       </c>
       <c r="E62" s="2">
-        <v>124.02873729314176</v>
+        <v>124.02873729314173</v>
       </c>
     </row>
     <row r="63">
@@ -1553,10 +1568,10 @@
         <v>2015</v>
       </c>
       <c r="D63" s="2">
-        <v>63.096850001600352</v>
+        <v>63.096850001600338</v>
       </c>
       <c r="E63" s="2">
-        <v>95.253253760130392</v>
+        <v>95.253253760130377</v>
       </c>
     </row>
     <row r="64">
@@ -1573,7 +1588,7 @@
         <v>67.298402962039859</v>
       </c>
       <c r="E64" s="2">
-        <v>136.09138427814997</v>
+        <v>136.09138427814995</v>
       </c>
     </row>
     <row r="65">
@@ -1587,7 +1602,7 @@
         <v>2017</v>
       </c>
       <c r="D65" s="2">
-        <v>77.910922958684793</v>
+        <v>77.910922958684807</v>
       </c>
       <c r="E65" s="2">
         <v>134.6241398568128</v>
@@ -1621,10 +1636,10 @@
         <v>2019</v>
       </c>
       <c r="D67" s="2">
-        <v>82.511839058747768</v>
+        <v>82.511839058747782</v>
       </c>
       <c r="E67" s="2">
-        <v>140.53768006006933</v>
+        <v>140.53768006006936</v>
       </c>
     </row>
     <row r="68">
@@ -1638,10 +1653,10 @@
         <v>2020</v>
       </c>
       <c r="D68" s="2">
-        <v>84.746575532747769</v>
+        <v>84.746575532747755</v>
       </c>
       <c r="E68" s="2">
-        <v>146.62608239079285</v>
+        <v>146.62608239079287</v>
       </c>
     </row>
     <row r="69">
@@ -1675,7 +1690,7 @@
         <v>65.485466952982989</v>
       </c>
       <c r="E70" s="2">
-        <v>153.94379226746625</v>
+        <v>153.94379226746622</v>
       </c>
     </row>
     <row r="71">
@@ -1689,10 +1704,10 @@
         <v>2023</v>
       </c>
       <c r="D71" s="2">
-        <v>67.995052411881929</v>
+        <v>67.9950524118819</v>
       </c>
       <c r="E71" s="2">
-        <v>144.77017142602574</v>
+        <v>144.77017142602571</v>
       </c>
     </row>
     <row r="72">
@@ -1709,7 +1724,7 @@
         <v>32.859156905523491</v>
       </c>
       <c r="E72" s="2">
-        <v>85.939465632385506</v>
+        <v>85.93946563238552</v>
       </c>
     </row>
     <row r="73">
@@ -1726,7 +1741,7 @@
         <v>31.537693052799</v>
       </c>
       <c r="E73" s="2">
-        <v>73.061416179947472</v>
+        <v>73.061416179947457</v>
       </c>
     </row>
     <row r="74">
@@ -1774,10 +1789,10 @@
         <v>2014</v>
       </c>
       <c r="D76" s="2">
-        <v>56.098523893632731</v>
+        <v>56.098523893632717</v>
       </c>
       <c r="E76" s="2">
-        <v>95.203378791033131</v>
+        <v>95.203378791033103</v>
       </c>
     </row>
     <row r="77">
@@ -1811,7 +1826,7 @@
         <v>51.79532335089624</v>
       </c>
       <c r="E78" s="2">
-        <v>100.53182582543312</v>
+        <v>100.53182582543315</v>
       </c>
     </row>
     <row r="79">
@@ -1842,10 +1857,10 @@
         <v>2018</v>
       </c>
       <c r="D80" s="2">
-        <v>58.275368982340389</v>
+        <v>58.275368982340382</v>
       </c>
       <c r="E80" s="2">
-        <v>106.84772812116829</v>
+        <v>106.84772812116833</v>
       </c>
     </row>
     <row r="81">
@@ -1859,7 +1874,7 @@
         <v>2019</v>
       </c>
       <c r="D81" s="2">
-        <v>68.357824785832051</v>
+        <v>68.357824785832065</v>
       </c>
       <c r="E81" s="2">
         <v>118.10145660973863</v>
@@ -1879,7 +1894,7 @@
         <v>62.987702944194631</v>
       </c>
       <c r="E82" s="2">
-        <v>116.77314767711917</v>
+        <v>116.7731476771192</v>
       </c>
     </row>
     <row r="83">
@@ -2301,13 +2316,13 @@
         <v>84</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2">
@@ -2438,7 +2453,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B11" s="1">
         <v>1.1160000000000001</v>
@@ -2452,7 +2467,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B12" s="1">
         <v>1.248</v>
@@ -2466,7 +2481,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B13" s="1">
         <v>1.264</v>
@@ -2480,7 +2495,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B14" s="1">
         <v>1.159</v>
@@ -2494,7 +2509,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B15" s="1">
         <v>1.218</v>
@@ -2528,18 +2543,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
         <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -2550,7 +2565,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
@@ -2561,7 +2576,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
         <v>35</v>
@@ -2572,7 +2587,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
         <v>36</v>
@@ -2583,18 +2598,18 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B8" t="s">
         <v>38</v>
@@ -2605,7 +2620,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
@@ -2616,7 +2631,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
         <v>40</v>
@@ -2627,7 +2642,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
         <v>41</v>
@@ -2638,29 +2653,29 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B12" t="s">
         <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
         <v>44</v>
@@ -2671,7 +2686,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
         <v>45</v>
@@ -2682,7 +2697,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B16" t="s">
         <v>46</v>
@@ -2693,7 +2708,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B17" t="s">
         <v>47</v>
@@ -2704,7 +2719,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B18" t="s">
         <v>48</v>
@@ -2747,7 +2762,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
         <v>84</v>
@@ -2756,36 +2771,36 @@
         <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="G2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
         <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
         <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G3" t="s">
         <v>74</v>
@@ -2793,22 +2808,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
         <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
         <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G4" t="s">
         <v>74</v>
@@ -2816,22 +2831,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
         <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E5" t="s">
         <v>74</v>
       </c>
       <c r="F5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="G5" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Briefing workflow step 1 draft completed
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
@@ -87,7 +87,7 @@
     <t>2023</t>
   </si>
   <si>
-    <t>2026-05-15</t>
+    <t>2026-08-03</t>
   </si>
   <si>
     <t>Data sheets, dataset metadata sheets, and variable metadata sheets</t>
@@ -576,7 +576,7 @@
         <v>95.221075283944316</v>
       </c>
       <c r="E2" s="2">
-        <v>129.84966844900714</v>
+        <v>129.84966844900708</v>
       </c>
     </row>
     <row r="3">
@@ -593,7 +593,7 @@
         <v>86.955464237230856</v>
       </c>
       <c r="E3" s="2">
-        <v>123.95548470731528</v>
+        <v>123.95548470731526</v>
       </c>
     </row>
     <row r="4">
@@ -610,7 +610,7 @@
         <v>83.958370647084877</v>
       </c>
       <c r="E4" s="2">
-        <v>125.98492039902337</v>
+        <v>125.98492039902339</v>
       </c>
     </row>
     <row r="5">
@@ -661,7 +661,7 @@
         <v>102.44156425394573</v>
       </c>
       <c r="E7" s="2">
-        <v>123.99215185512165</v>
+        <v>123.99215185512162</v>
       </c>
     </row>
     <row r="8">
@@ -678,7 +678,7 @@
         <v>122.32534407494403</v>
       </c>
       <c r="E8" s="2">
-        <v>154.40773688908658</v>
+        <v>154.40773688908661</v>
       </c>
     </row>
     <row r="9">
@@ -692,7 +692,7 @@
         <v>2017</v>
       </c>
       <c r="D9" s="2">
-        <v>113.46297582983942</v>
+        <v>113.46297582983944</v>
       </c>
       <c r="E9" s="2">
         <v>134.09629973602568</v>
@@ -712,7 +712,7 @@
         <v>107.65095729890692</v>
       </c>
       <c r="E10" s="2">
-        <v>134.91772827836096</v>
+        <v>134.91772827836098</v>
       </c>
     </row>
     <row r="11">
@@ -729,7 +729,7 @@
         <v>119.09170030342358</v>
       </c>
       <c r="E11" s="2">
-        <v>144.1067785803204</v>
+        <v>144.10677858032042</v>
       </c>
     </row>
     <row r="12">
@@ -743,7 +743,7 @@
         <v>2020</v>
       </c>
       <c r="D12" s="2">
-        <v>110.10122741163116</v>
+        <v>110.10122741163111</v>
       </c>
       <c r="E12" s="2">
         <v>136.24593394275945</v>
@@ -763,7 +763,7 @@
         <v>98.03239321958435</v>
       </c>
       <c r="E13" s="2">
-        <v>126.94754679620044</v>
+        <v>126.94754679620041</v>
       </c>
     </row>
     <row r="14">
@@ -777,7 +777,7 @@
         <v>2022</v>
       </c>
       <c r="D14" s="2">
-        <v>106.1756868524164</v>
+        <v>106.17568685241639</v>
       </c>
       <c r="E14" s="2">
         <v>136.01723072341716</v>
@@ -797,7 +797,7 @@
         <v>111.89575841376259</v>
       </c>
       <c r="E15" s="2">
-        <v>140.99776699415861</v>
+        <v>140.99776699415864</v>
       </c>
     </row>
     <row r="16">
@@ -845,7 +845,7 @@
         <v>2012</v>
       </c>
       <c r="D18" s="2">
-        <v>114.55911018767614</v>
+        <v>114.55911018767617</v>
       </c>
       <c r="E18" s="2">
         <v>150.37591834701553</v>
@@ -862,7 +862,7 @@
         <v>2013</v>
       </c>
       <c r="D19" s="2">
-        <v>153.29967899492223</v>
+        <v>153.29967899492226</v>
       </c>
       <c r="E19" s="2">
         <v>188.36042775237485</v>
@@ -879,10 +879,10 @@
         <v>2014</v>
       </c>
       <c r="D20" s="2">
-        <v>125.33096468512296</v>
+        <v>125.33096468512295</v>
       </c>
       <c r="E20" s="2">
-        <v>151.69288037849714</v>
+        <v>151.69288037849716</v>
       </c>
     </row>
     <row r="21">
@@ -896,10 +896,10 @@
         <v>2015</v>
       </c>
       <c r="D21" s="2">
-        <v>126.40360469611636</v>
+        <v>126.40360469611637</v>
       </c>
       <c r="E21" s="2">
-        <v>147.36292080522935</v>
+        <v>147.36292080522929</v>
       </c>
     </row>
     <row r="22">
@@ -916,7 +916,7 @@
         <v>141.21050447640192</v>
       </c>
       <c r="E22" s="2">
-        <v>178.69433588102012</v>
+        <v>178.69433588102018</v>
       </c>
     </row>
     <row r="23">
@@ -930,7 +930,7 @@
         <v>2017</v>
       </c>
       <c r="D23" s="2">
-        <v>137.78899295395163</v>
+        <v>137.78899295395166</v>
       </c>
       <c r="E23" s="2">
         <v>161.52816429751982</v>
@@ -981,7 +981,7 @@
         <v>2020</v>
       </c>
       <c r="D26" s="2">
-        <v>139.3940110249097</v>
+        <v>139.39401102490973</v>
       </c>
       <c r="E26" s="2">
         <v>169.28851560092858</v>
@@ -1015,7 +1015,7 @@
         <v>2022</v>
       </c>
       <c r="D28" s="2">
-        <v>135.55051913987518</v>
+        <v>135.55051913987521</v>
       </c>
       <c r="E28" s="2">
         <v>187.12143427741455</v>
@@ -1035,7 +1035,7 @@
         <v>153.96482802987171</v>
       </c>
       <c r="E29" s="2">
-        <v>197.85764950643468</v>
+        <v>197.85764950643474</v>
       </c>
     </row>
     <row r="30">
@@ -1052,7 +1052,7 @@
         <v>108.19131887864872</v>
       </c>
       <c r="E30" s="2">
-        <v>143.76442335625933</v>
+        <v>143.7644233562593</v>
       </c>
     </row>
     <row r="31">
@@ -1083,10 +1083,10 @@
         <v>2012</v>
       </c>
       <c r="D32" s="2">
-        <v>97.496314274191263</v>
+        <v>97.496314274191249</v>
       </c>
       <c r="E32" s="2">
-        <v>137.91417726388366</v>
+        <v>137.91417726388363</v>
       </c>
     </row>
     <row r="33">
@@ -1100,10 +1100,10 @@
         <v>2013</v>
       </c>
       <c r="D33" s="2">
-        <v>132.43103487164564</v>
+        <v>132.43103487164561</v>
       </c>
       <c r="E33" s="2">
-        <v>165.76438905854454</v>
+        <v>165.76438905854451</v>
       </c>
     </row>
     <row r="34">
@@ -1117,10 +1117,10 @@
         <v>2014</v>
       </c>
       <c r="D34" s="2">
-        <v>115.29448083495105</v>
+        <v>115.2944808349511</v>
       </c>
       <c r="E34" s="2">
-        <v>137.41944314066936</v>
+        <v>137.41944314066933</v>
       </c>
     </row>
     <row r="35">
@@ -1134,7 +1134,7 @@
         <v>2015</v>
       </c>
       <c r="D35" s="2">
-        <v>113.84661645574478</v>
+        <v>113.84661645574481</v>
       </c>
       <c r="E35" s="2">
         <v>135.50382164638725</v>
@@ -1154,7 +1154,7 @@
         <v>131.85208906168819</v>
       </c>
       <c r="E36" s="2">
-        <v>166.16480818173733</v>
+        <v>166.1648081817373</v>
       </c>
     </row>
     <row r="37">
@@ -1185,10 +1185,10 @@
         <v>2018</v>
       </c>
       <c r="D38" s="2">
-        <v>124.24670561488773</v>
+        <v>124.24670561488777</v>
       </c>
       <c r="E38" s="2">
-        <v>152.4328094642992</v>
+        <v>152.43280946429917</v>
       </c>
     </row>
     <row r="39">
@@ -1253,10 +1253,10 @@
         <v>2022</v>
       </c>
       <c r="D42" s="2">
-        <v>119.5777561015874</v>
+        <v>119.57775610158743</v>
       </c>
       <c r="E42" s="2">
-        <v>158.71716158231376</v>
+        <v>158.71716158231379</v>
       </c>
     </row>
     <row r="43">
@@ -1307,7 +1307,7 @@
         <v>20.736462077997842</v>
       </c>
       <c r="E45" s="2">
-        <v>50.749670433101471</v>
+        <v>50.7496704331015</v>
       </c>
     </row>
     <row r="46">
@@ -1324,7 +1324,7 @@
         <v>40.861820365951232</v>
       </c>
       <c r="E46" s="2">
-        <v>80.862069789296101</v>
+        <v>80.862069789296072</v>
       </c>
     </row>
     <row r="47">
@@ -1355,7 +1355,7 @@
         <v>2014</v>
       </c>
       <c r="D48" s="2">
-        <v>44.404040284993002</v>
+        <v>44.404040284992988</v>
       </c>
       <c r="E48" s="2">
         <v>72.28720220218996</v>
@@ -1375,7 +1375,7 @@
         <v>40.436169377381504</v>
       </c>
       <c r="E49" s="2">
-        <v>60.611178070548441</v>
+        <v>60.611178070548434</v>
       </c>
     </row>
     <row r="50">
@@ -1477,7 +1477,7 @@
         <v>34.016850240943995</v>
       </c>
       <c r="E55" s="2">
-        <v>76.494922085252966</v>
+        <v>76.494922085252981</v>
       </c>
     </row>
     <row r="56">
@@ -1494,7 +1494,7 @@
         <v>38.830144120011511</v>
       </c>
       <c r="E56" s="2">
-        <v>87.948672510579144</v>
+        <v>87.948672510579129</v>
       </c>
     </row>
     <row r="57">
@@ -1528,7 +1528,7 @@
         <v>39.871986215342048</v>
       </c>
       <c r="E58" s="2">
-        <v>100.25991604723204</v>
+        <v>100.25991604723207</v>
       </c>
     </row>
     <row r="59">
@@ -1542,7 +1542,7 @@
         <v>2011</v>
       </c>
       <c r="D59" s="2">
-        <v>44.350439311810732</v>
+        <v>44.350439311810746</v>
       </c>
       <c r="E59" s="2">
         <v>101.00182079274421</v>
@@ -1562,7 +1562,7 @@
         <v>53.267849983925743</v>
       </c>
       <c r="E60" s="2">
-        <v>119.72367489464595</v>
+        <v>119.72367489464597</v>
       </c>
     </row>
     <row r="61">
@@ -1576,7 +1576,7 @@
         <v>2013</v>
       </c>
       <c r="D61" s="2">
-        <v>51.632423592605932</v>
+        <v>51.632423592605918</v>
       </c>
       <c r="E61" s="2">
         <v>111.52272891322129</v>
@@ -1630,7 +1630,7 @@
         <v>67.298402962039859</v>
       </c>
       <c r="E64" s="2">
-        <v>136.09138427814995</v>
+        <v>136.09138427814997</v>
       </c>
     </row>
     <row r="65">
@@ -1644,7 +1644,7 @@
         <v>2017</v>
       </c>
       <c r="D65" s="2">
-        <v>77.910922958684793</v>
+        <v>77.910922958684807</v>
       </c>
       <c r="E65" s="2">
         <v>134.6241398568128</v>
@@ -1661,7 +1661,7 @@
         <v>2018</v>
       </c>
       <c r="D66" s="2">
-        <v>79.962100676298675</v>
+        <v>79.962100676298689</v>
       </c>
       <c r="E66" s="2">
         <v>142.28837093119805</v>
@@ -1681,7 +1681,7 @@
         <v>82.511839058747768</v>
       </c>
       <c r="E67" s="2">
-        <v>140.53768006006933</v>
+        <v>140.53768006006936</v>
       </c>
     </row>
     <row r="68">
@@ -1695,10 +1695,10 @@
         <v>2020</v>
       </c>
       <c r="D68" s="2">
-        <v>84.746575532747769</v>
+        <v>84.746575532747755</v>
       </c>
       <c r="E68" s="2">
-        <v>146.62608239079287</v>
+        <v>146.62608239079285</v>
       </c>
     </row>
     <row r="69">
@@ -1732,7 +1732,7 @@
         <v>65.485466952983003</v>
       </c>
       <c r="E70" s="2">
-        <v>153.94379226746625</v>
+        <v>153.94379226746622</v>
       </c>
     </row>
     <row r="71">
@@ -1746,10 +1746,10 @@
         <v>2023</v>
       </c>
       <c r="D71" s="2">
-        <v>67.995052411881929</v>
+        <v>67.9950524118819</v>
       </c>
       <c r="E71" s="2">
-        <v>144.77017142602571</v>
+        <v>144.77017142602574</v>
       </c>
     </row>
     <row r="72">
@@ -1800,7 +1800,7 @@
         <v>46.493243333067454</v>
       </c>
       <c r="E74" s="2">
-        <v>98.372077995995952</v>
+        <v>98.372077995995923</v>
       </c>
     </row>
     <row r="75">
@@ -1817,7 +1817,7 @@
         <v>38.308254895032519</v>
       </c>
       <c r="E75" s="2">
-        <v>84.395112720829488</v>
+        <v>84.395112720829474</v>
       </c>
     </row>
     <row r="76">
@@ -1848,7 +1848,7 @@
         <v>2015</v>
       </c>
       <c r="D77" s="2">
-        <v>51.214620843783848</v>
+        <v>51.214620843783862</v>
       </c>
       <c r="E77" s="2">
         <v>76.650630627800695</v>
@@ -1885,7 +1885,7 @@
         <v>64.277420152441564</v>
       </c>
       <c r="E79" s="2">
-        <v>104.93675001582747</v>
+        <v>104.93675001582744</v>
       </c>
     </row>
     <row r="80">
@@ -1919,7 +1919,7 @@
         <v>68.357824785832051</v>
       </c>
       <c r="E81" s="2">
-        <v>118.10145660973863</v>
+        <v>118.10145660973866</v>
       </c>
     </row>
     <row r="82">
@@ -1933,7 +1933,7 @@
         <v>2020</v>
       </c>
       <c r="D82" s="2">
-        <v>62.987702944194645</v>
+        <v>62.987702944194631</v>
       </c>
       <c r="E82" s="2">
         <v>116.77314767711917</v>
@@ -1953,7 +1953,7 @@
         <v>44.774283406883086</v>
       </c>
       <c r="E83" s="2">
-        <v>97.269587462146589</v>
+        <v>97.269587462146575</v>
       </c>
     </row>
     <row r="84">
@@ -1970,7 +1970,7 @@
         <v>50.910595133117283</v>
       </c>
       <c r="E84" s="2">
-        <v>116.48295164884803</v>
+        <v>116.48295164884804</v>
       </c>
     </row>
     <row r="85">
@@ -1984,7 +1984,7 @@
         <v>2023</v>
       </c>
       <c r="D85" s="2">
-        <v>52.325903563904532</v>
+        <v>52.325903563904518</v>
       </c>
       <c r="E85" s="2">
         <v>115.56635726330089</v>

</xml_diff>

<commit_message>
Update to LoS analytics. Re-published v1 briefings
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_incidence_2023_v1/workbook/bnr_cvd_incidence_2023_v1.xlsx
@@ -87,7 +87,7 @@
     <t>2023</t>
   </si>
   <si>
-    <t>2026-08-07</t>
+    <t>2026-08-13</t>
   </si>
   <si>
     <t>Data sheets, dataset metadata sheets, and variable metadata sheets</t>
@@ -1209,10 +1209,10 @@
         <v>2010</v>
       </c>
       <c r="D2" s="2">
-        <v>95.221075283944316</v>
+        <v>95.22107528394433</v>
       </c>
       <c r="E2" s="2">
-        <v>129.84966844900714</v>
+        <v>129.84966844900708</v>
       </c>
     </row>
     <row r="3">
@@ -1246,7 +1246,7 @@
         <v>83.958370647084877</v>
       </c>
       <c r="E4" s="2">
-        <v>125.98492039902339</v>
+        <v>125.98492039902337</v>
       </c>
     </row>
     <row r="5">
@@ -1260,10 +1260,10 @@
         <v>2013</v>
       </c>
       <c r="D5" s="2">
-        <v>115.84453460256653</v>
+        <v>115.84453460256651</v>
       </c>
       <c r="E5" s="2">
-        <v>148.16213688134337</v>
+        <v>148.16213688134334</v>
       </c>
     </row>
     <row r="6">
@@ -1294,7 +1294,7 @@
         <v>2015</v>
       </c>
       <c r="D7" s="2">
-        <v>102.44156425394576</v>
+        <v>102.44156425394573</v>
       </c>
       <c r="E7" s="2">
         <v>123.99215185512162</v>
@@ -1314,7 +1314,7 @@
         <v>122.03745291848145</v>
       </c>
       <c r="E8" s="2">
-        <v>154.11984573262399</v>
+        <v>154.11984573262401</v>
       </c>
     </row>
     <row r="9">
@@ -1345,10 +1345,10 @@
         <v>2018</v>
       </c>
       <c r="D10" s="2">
-        <v>107.65095729890692</v>
+        <v>107.65095729890695</v>
       </c>
       <c r="E10" s="2">
-        <v>134.06963208597617</v>
+        <v>134.0696320859762</v>
       </c>
     </row>
     <row r="11">
@@ -1365,7 +1365,7 @@
         <v>119.09170030342358</v>
       </c>
       <c r="E11" s="2">
-        <v>144.1067785803204</v>
+        <v>144.10677858032042</v>
       </c>
     </row>
     <row r="12">
@@ -1379,10 +1379,10 @@
         <v>2020</v>
       </c>
       <c r="D12" s="2">
-        <v>110.1012274116311</v>
+        <v>110.10122741163111</v>
       </c>
       <c r="E12" s="2">
-        <v>136.24593394275945</v>
+        <v>136.24593394275942</v>
       </c>
     </row>
     <row r="13">
@@ -1396,7 +1396,7 @@
         <v>2021</v>
       </c>
       <c r="D13" s="2">
-        <v>98.032393219584364</v>
+        <v>98.03239321958435</v>
       </c>
       <c r="E13" s="2">
         <v>126.94754679620046</v>
@@ -1416,7 +1416,7 @@
         <v>106.17568685241636</v>
       </c>
       <c r="E14" s="2">
-        <v>136.01723072341716</v>
+        <v>136.01723072341719</v>
       </c>
     </row>
     <row r="15">
@@ -1467,7 +1467,7 @@
         <v>109.30850739434268</v>
       </c>
       <c r="E17" s="2">
-        <v>155.36787412863708</v>
+        <v>155.36787412863711</v>
       </c>
     </row>
     <row r="18">
@@ -1481,7 +1481,7 @@
         <v>2012</v>
       </c>
       <c r="D18" s="2">
-        <v>114.55911018767614</v>
+        <v>114.55911018767617</v>
       </c>
       <c r="E18" s="2">
         <v>150.37591834701553</v>
@@ -1515,10 +1515,10 @@
         <v>2014</v>
       </c>
       <c r="D20" s="2">
-        <v>125.33096468512295</v>
+        <v>125.33096468512299</v>
       </c>
       <c r="E20" s="2">
-        <v>151.69288037849714</v>
+        <v>151.69288037849719</v>
       </c>
     </row>
     <row r="21">
@@ -1532,10 +1532,10 @@
         <v>2015</v>
       </c>
       <c r="D21" s="2">
-        <v>126.40360469611636</v>
+        <v>126.40360469611637</v>
       </c>
       <c r="E21" s="2">
-        <v>147.36292080522932</v>
+        <v>147.36292080522929</v>
       </c>
     </row>
     <row r="22">
@@ -1549,10 +1549,10 @@
         <v>2016</v>
       </c>
       <c r="D22" s="2">
-        <v>141.21050447640192</v>
+        <v>141.21050447640189</v>
       </c>
       <c r="E22" s="2">
-        <v>178.11434501761218</v>
+        <v>178.11434501761221</v>
       </c>
     </row>
     <row r="23">
@@ -1583,7 +1583,7 @@
         <v>2018</v>
       </c>
       <c r="D24" s="2">
-        <v>143.09130434286232</v>
+        <v>143.09130434286234</v>
       </c>
       <c r="E24" s="2">
         <v>170.30983149870136</v>
@@ -1600,10 +1600,10 @@
         <v>2019</v>
       </c>
       <c r="D25" s="2">
-        <v>152.20620714994263</v>
+        <v>152.20620714994266</v>
       </c>
       <c r="E25" s="2">
-        <v>183.10483234403156</v>
+        <v>183.10483234403154</v>
       </c>
     </row>
     <row r="26">
@@ -1634,10 +1634,10 @@
         <v>2021</v>
       </c>
       <c r="D27" s="2">
-        <v>133.04510412862652</v>
+        <v>133.04510412862649</v>
       </c>
       <c r="E27" s="2">
-        <v>166.87172048037419</v>
+        <v>166.87172048037422</v>
       </c>
     </row>
     <row r="28">
@@ -1651,10 +1651,10 @@
         <v>2022</v>
       </c>
       <c r="D28" s="2">
-        <v>135.55051913987523</v>
+        <v>135.55051913987518</v>
       </c>
       <c r="E28" s="2">
-        <v>187.12143427741452</v>
+        <v>187.12143427741455</v>
       </c>
     </row>
     <row r="29">
@@ -1685,10 +1685,10 @@
         <v>2010</v>
       </c>
       <c r="D30" s="2">
-        <v>108.19131887864872</v>
+        <v>108.1913188786487</v>
       </c>
       <c r="E30" s="2">
-        <v>143.7644233562593</v>
+        <v>143.76442335625933</v>
       </c>
     </row>
     <row r="31">
@@ -1702,7 +1702,7 @@
         <v>2011</v>
       </c>
       <c r="D31" s="2">
-        <v>97.059790074554712</v>
+        <v>97.059790074554726</v>
       </c>
       <c r="E31" s="2">
         <v>138.75412658257849</v>
@@ -1719,7 +1719,7 @@
         <v>2012</v>
       </c>
       <c r="D32" s="2">
-        <v>97.496314274191263</v>
+        <v>97.496314274191249</v>
       </c>
       <c r="E32" s="2">
         <v>137.91417726388366</v>
@@ -1736,10 +1736,10 @@
         <v>2013</v>
       </c>
       <c r="D33" s="2">
-        <v>132.43103487164558</v>
+        <v>132.43103487164564</v>
       </c>
       <c r="E33" s="2">
-        <v>165.76438905854451</v>
+        <v>165.76438905854454</v>
       </c>
     </row>
     <row r="34">
@@ -1753,10 +1753,10 @@
         <v>2014</v>
       </c>
       <c r="D34" s="2">
-        <v>115.29448083495105</v>
+        <v>115.29448083495107</v>
       </c>
       <c r="E34" s="2">
-        <v>137.41944314066933</v>
+        <v>137.41944314066936</v>
       </c>
     </row>
     <row r="35">
@@ -1804,10 +1804,10 @@
         <v>2017</v>
       </c>
       <c r="D37" s="2">
-        <v>123.9723359281213</v>
+        <v>123.97233592812131</v>
       </c>
       <c r="E37" s="2">
-        <v>146.31769719669242</v>
+        <v>146.31769719669236</v>
       </c>
     </row>
     <row r="38">
@@ -1821,10 +1821,10 @@
         <v>2018</v>
       </c>
       <c r="D38" s="2">
-        <v>124.24670561488777</v>
+        <v>124.24670561488776</v>
       </c>
       <c r="E38" s="2">
-        <v>151.30527838081784</v>
+        <v>151.30527838081781</v>
       </c>
     </row>
     <row r="39">
@@ -1838,7 +1838,7 @@
         <v>2019</v>
       </c>
       <c r="D39" s="2">
-        <v>135.14000336761538</v>
+        <v>135.14000336761541</v>
       </c>
       <c r="E39" s="2">
         <v>162.50172387540604</v>
@@ -1858,7 +1858,7 @@
         <v>124.30445543196635</v>
       </c>
       <c r="E40" s="2">
-        <v>152.29672324055019</v>
+        <v>152.29672324055017</v>
       </c>
     </row>
     <row r="41">
@@ -1889,7 +1889,7 @@
         <v>2022</v>
       </c>
       <c r="D42" s="2">
-        <v>119.57775610158743</v>
+        <v>119.5777561015874</v>
       </c>
       <c r="E42" s="2">
         <v>158.71716158231376</v>
@@ -1943,7 +1943,7 @@
         <v>20.736462077997842</v>
       </c>
       <c r="E45" s="2">
-        <v>50.7496704331015</v>
+        <v>50.749670433101471</v>
       </c>
     </row>
     <row r="46">
@@ -1960,7 +1960,7 @@
         <v>40.861820365951232</v>
       </c>
       <c r="E46" s="2">
-        <v>80.862069789296101</v>
+        <v>80.862069789296072</v>
       </c>
     </row>
     <row r="47">
@@ -1991,7 +1991,7 @@
         <v>2014</v>
       </c>
       <c r="D48" s="2">
-        <v>44.404040284992988</v>
+        <v>44.404040284993002</v>
       </c>
       <c r="E48" s="2">
         <v>72.28720220218996</v>
@@ -2011,7 +2011,7 @@
         <v>40.436169377381504</v>
       </c>
       <c r="E49" s="2">
-        <v>60.611178070548419</v>
+        <v>60.611178070548434</v>
       </c>
     </row>
     <row r="50">
@@ -2076,7 +2076,7 @@
         <v>2019</v>
       </c>
       <c r="D53" s="2">
-        <v>55.358582369177711</v>
+        <v>55.358582369177697</v>
       </c>
       <c r="E53" s="2">
         <v>97.621168412514152</v>
@@ -2096,7 +2096,7 @@
         <v>45.543953356423003</v>
       </c>
       <c r="E54" s="2">
-        <v>91.141458171020332</v>
+        <v>91.141458171020347</v>
       </c>
     </row>
     <row r="55">
@@ -2113,7 +2113,7 @@
         <v>34.016850240943995</v>
       </c>
       <c r="E55" s="2">
-        <v>76.494922085252966</v>
+        <v>76.494922085252981</v>
       </c>
     </row>
     <row r="56">
@@ -2130,7 +2130,7 @@
         <v>38.830144120011511</v>
       </c>
       <c r="E56" s="2">
-        <v>87.948672510579144</v>
+        <v>87.948672510579129</v>
       </c>
     </row>
     <row r="57">
@@ -2147,7 +2147,7 @@
         <v>38.436967798230711</v>
       </c>
       <c r="E57" s="2">
-        <v>89.923140516683503</v>
+        <v>89.923140516683517</v>
       </c>
     </row>
     <row r="58">
@@ -2178,7 +2178,7 @@
         <v>2011</v>
       </c>
       <c r="D59" s="2">
-        <v>44.350439311810746</v>
+        <v>44.35043931181076</v>
       </c>
       <c r="E59" s="2">
         <v>101.00182079274421</v>
@@ -2195,7 +2195,7 @@
         <v>2012</v>
       </c>
       <c r="D60" s="2">
-        <v>53.267849983925743</v>
+        <v>53.267849983925771</v>
       </c>
       <c r="E60" s="2">
         <v>119.72367489464595</v>
@@ -2212,10 +2212,10 @@
         <v>2013</v>
       </c>
       <c r="D61" s="2">
-        <v>51.632423592605932</v>
+        <v>51.632423592605918</v>
       </c>
       <c r="E61" s="2">
-        <v>111.52272891322129</v>
+        <v>111.52272891322126</v>
       </c>
     </row>
     <row r="62">
@@ -2249,7 +2249,7 @@
         <v>63.096850001600352</v>
       </c>
       <c r="E63" s="2">
-        <v>95.253253760130392</v>
+        <v>95.253253760130406</v>
       </c>
     </row>
     <row r="64">
@@ -2280,7 +2280,7 @@
         <v>2017</v>
       </c>
       <c r="D65" s="2">
-        <v>77.910922958684807</v>
+        <v>77.910922958684793</v>
       </c>
       <c r="E65" s="2">
         <v>134.6241398568128</v>
@@ -2314,10 +2314,10 @@
         <v>2019</v>
       </c>
       <c r="D67" s="2">
-        <v>82.511839058747768</v>
+        <v>82.511839058747796</v>
       </c>
       <c r="E67" s="2">
-        <v>140.53768006006942</v>
+        <v>140.53768006006936</v>
       </c>
     </row>
     <row r="68">
@@ -2351,7 +2351,7 @@
         <v>57.16647908257449</v>
       </c>
       <c r="E69" s="2">
-        <v>121.96504986319471</v>
+        <v>121.96504986319472</v>
       </c>
     </row>
     <row r="70">
@@ -2382,7 +2382,7 @@
         <v>2023</v>
       </c>
       <c r="D71" s="2">
-        <v>67.995052411881915</v>
+        <v>67.995052411881929</v>
       </c>
       <c r="E71" s="2">
         <v>144.77017142602571</v>
@@ -2402,7 +2402,7 @@
         <v>32.859156905523491</v>
       </c>
       <c r="E72" s="2">
-        <v>85.93946563238552</v>
+        <v>85.939465632385506</v>
       </c>
     </row>
     <row r="73">
@@ -2436,7 +2436,7 @@
         <v>46.493243333067454</v>
       </c>
       <c r="E74" s="2">
-        <v>98.372077995995952</v>
+        <v>98.372077995995923</v>
       </c>
     </row>
     <row r="75">
@@ -2453,7 +2453,7 @@
         <v>38.308254895032519</v>
       </c>
       <c r="E75" s="2">
-        <v>84.395112720829488</v>
+        <v>84.395112720829474</v>
       </c>
     </row>
     <row r="76">
@@ -2467,10 +2467,10 @@
         <v>2014</v>
       </c>
       <c r="D76" s="2">
-        <v>56.098523893632731</v>
+        <v>56.098523893632738</v>
       </c>
       <c r="E76" s="2">
-        <v>95.203378791033103</v>
+        <v>95.203378791033117</v>
       </c>
     </row>
     <row r="77">
@@ -2484,7 +2484,7 @@
         <v>2015</v>
       </c>
       <c r="D77" s="2">
-        <v>51.214620843783848</v>
+        <v>51.214620843783862</v>
       </c>
       <c r="E77" s="2">
         <v>76.650630627800695</v>
@@ -2518,7 +2518,7 @@
         <v>2017</v>
       </c>
       <c r="D79" s="2">
-        <v>64.277420152441564</v>
+        <v>64.277420152441579</v>
       </c>
       <c r="E79" s="2">
         <v>104.93675001582744</v>
@@ -2535,10 +2535,10 @@
         <v>2018</v>
       </c>
       <c r="D80" s="2">
-        <v>58.275368982340368</v>
+        <v>58.275368982340382</v>
       </c>
       <c r="E80" s="2">
-        <v>106.8477281211683</v>
+        <v>106.84772812116833</v>
       </c>
     </row>
     <row r="81">
@@ -2606,7 +2606,7 @@
         <v>50.910595133117283</v>
       </c>
       <c r="E84" s="2">
-        <v>116.48295164884803</v>
+        <v>116.48295164884804</v>
       </c>
     </row>
     <row r="85">
@@ -2620,7 +2620,7 @@
         <v>2023</v>
       </c>
       <c r="D85" s="2">
-        <v>52.325903563904532</v>
+        <v>52.325903563904518</v>
       </c>
       <c r="E85" s="2">
         <v>115.5663572633009</v>

</xml_diff>